<commit_message>
refactor: change bg color to a darker shade
</commit_message>
<xml_diff>
--- a/tests/128/128.xlsx
+++ b/tests/128/128.xlsx
@@ -1,58 +1,63 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="124">
-  <si>
-    <t>Kobeni Hour</t>
-  </si>
-  <si>
-    <t>YYY Y YNN N NYY Y</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
+  <si>
+    <t xml:space="preserve">Kobeni Hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYY Y YNN N NYY Y</t>
   </si>
   <si>
     <t>Nomad</t>
   </si>
   <si>
-    <t>N Y N N  N N N N  N Y N N</t>
+    <t xml:space="preserve">N Y N N  N N N N  N Y N N</t>
   </si>
   <si>
     <t>Golden</t>
   </si>
   <si>
-    <t>YYNY YNNN NNYN</t>
+    <t xml:space="preserve">YYNY YNNN NNYN</t>
   </si>
   <si>
     <t>naian77</t>
   </si>
   <si>
-    <t>YYNN YNNN YNYN</t>
-  </si>
-  <si>
-    <t>Daniel Gacitua</t>
-  </si>
-  <si>
-    <t>YYNY NNNN YYYN</t>
-  </si>
-  <si>
-    <t>Urek vs Macseth | Rolo</t>
-  </si>
-  <si>
-    <t>NNNN NNNN NYYN</t>
-  </si>
-  <si>
-    <t>Po Bi D. Au</t>
-  </si>
-  <si>
-    <t>NYNY YNNN NYYN</t>
+    <t xml:space="preserve">YYNN YNNN YNYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daniel Gacitua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYNY NNNN YYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Urek vs Macseth | Rolo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNNN NNNN NYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Po Bi D. Au</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYNY YNNN NYYN</t>
   </si>
   <si>
     <t>LaFa</t>
@@ -61,199 +66,199 @@
     <t>Jain_friend69</t>
   </si>
   <si>
-    <t>Y Y N N    Y N N Y      Y Y N Y</t>
+    <t xml:space="preserve">Y Y N N    Y N N Y      Y Y N Y</t>
   </si>
   <si>
     <t>Kanika_em</t>
   </si>
   <si>
-    <t>YYNY NNNN NNYN</t>
+    <t xml:space="preserve">YYNY NNNN NNYN</t>
   </si>
   <si>
     <t>hajro</t>
   </si>
   <si>
-    <t>YYYN YNNY NYYN</t>
-  </si>
-  <si>
-    <t>Peak-A-Boo | FATE</t>
-  </si>
-  <si>
-    <t>YNNN YNNY NYYN</t>
+    <t xml:space="preserve">YYYN YNNY NYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peak-A-Boo | FATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YNNN YNNY NYYN</t>
   </si>
   <si>
     <t>Muddy</t>
   </si>
   <si>
-    <t>YYYN YNNY YYYN</t>
+    <t xml:space="preserve">YYYN YNNY YYYN</t>
   </si>
   <si>
     <t>Karneval</t>
   </si>
   <si>
-    <t>YYNN YNNN YYYN</t>
-  </si>
-  <si>
-    <t>Ranker BaamZahard</t>
-  </si>
-  <si>
-    <t>YYNN NNNN NNYY</t>
+    <t xml:space="preserve">YYNN YNNN YYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ranker BaamZahard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYNN NNNN NNYY</t>
   </si>
   <si>
     <t>Ozymanbruh</t>
   </si>
   <si>
-    <t>YNYY YYNN YYYN</t>
-  </si>
-  <si>
-    <t>Griot | ♾</t>
-  </si>
-  <si>
-    <t>NNYN YNNN NYNY</t>
+    <t xml:space="preserve">YNYY YYNN YYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Griot | ♾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNYN YNNN NYNY</t>
   </si>
   <si>
     <t>malts</t>
   </si>
   <si>
-    <t>YYYN NNNN NYYY</t>
+    <t xml:space="preserve">YYYN NNNN NYYY</t>
   </si>
   <si>
     <t>Eggroll6996</t>
   </si>
   <si>
-    <t>NYNN NNNN NYYN</t>
+    <t xml:space="preserve">NYNN NNNN NYYN</t>
   </si>
   <si>
     <t>Hatikva</t>
   </si>
   <si>
-    <t>YYNN YNYN NYYN</t>
+    <t xml:space="preserve">YYNN YNYN NYYN</t>
   </si>
   <si>
     <t>Eiheir</t>
   </si>
   <si>
-    <t>YYN Y YNN N NYY Y</t>
-  </si>
-  <si>
-    <t>colorless june</t>
-  </si>
-  <si>
-    <t>NNYY YNYN NYNN</t>
+    <t xml:space="preserve">YYN Y YNN N NYY Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">colorless june</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNYY YNYN NYNN</t>
   </si>
   <si>
     <t>RajaBranco</t>
   </si>
   <si>
-    <t>YYNN YNNN NYYN</t>
+    <t xml:space="preserve">YYNN YNNN NYYN</t>
   </si>
   <si>
     <t>Saint</t>
   </si>
   <si>
-    <t>YYYN YNYY  YNYN</t>
-  </si>
-  <si>
-    <t>Best girl For sure</t>
+    <t xml:space="preserve">YYYN YNYY  YNYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best girl For sure</t>
   </si>
   <si>
     <t>Headon's🍆Heaven</t>
   </si>
   <si>
-    <t>NYYN YNYY NYNN</t>
-  </si>
-  <si>
-    <t>Rodeosquad 👑| Son Of Ari</t>
-  </si>
-  <si>
-    <t>YNNY YNNN NYYN</t>
+    <t xml:space="preserve">NYYN YNYY NYNN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rodeosquad 👑| Son Of Ari</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YNNY YNNN NYYN</t>
   </si>
   <si>
     <t>Platon</t>
   </si>
   <si>
-    <t>YYNY YNNN NYYN</t>
-  </si>
-  <si>
-    <t>Thien | thicc thighs save lives</t>
-  </si>
-  <si>
-    <t>YYNN NNNN NYYN</t>
-  </si>
-  <si>
-    <t>Amr Ahmed | Jinsung supremacy |</t>
-  </si>
-  <si>
-    <t>YYYY YNYY YYYY</t>
-  </si>
-  <si>
-    <t>Jinsung fanboy</t>
-  </si>
-  <si>
-    <t>NNNN NNNN NNNN</t>
+    <t xml:space="preserve">YYNY YNNN NYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thien | thicc thighs save lives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYNN NNNN NYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amr Ahmed | Jinsung supremacy |</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYYY YNYY YYYY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jinsung fanboy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNNN NNNN NNNN</t>
   </si>
   <si>
     <t>SirLordBoss</t>
   </si>
   <si>
-    <t>YYYY YYYY NYNN</t>
+    <t xml:space="preserve">YYYY YYYY NYNN</t>
   </si>
   <si>
     <t>Sathya</t>
   </si>
   <si>
-    <t>YYYY YYYY YYYY</t>
+    <t xml:space="preserve">YYYY YYYY YYYY</t>
   </si>
   <si>
     <t>Naronu</t>
   </si>
   <si>
-    <t>Y Y N N Y N N Y Y N Y N</t>
+    <t xml:space="preserve">Y Y N N Y N N Y Y N Y N</t>
   </si>
   <si>
     <t>Popcorn</t>
   </si>
   <si>
-    <t>NNNN YNNN YYYN</t>
+    <t xml:space="preserve">NNNN YNNN YYYN</t>
   </si>
   <si>
     <t>Lopobiasimp</t>
   </si>
   <si>
-    <t>NNNY YNYN NYNN</t>
+    <t xml:space="preserve">NNNY YNYN NYNN</t>
   </si>
   <si>
     <t>RTSK0929</t>
   </si>
   <si>
-    <t>N N Y N N N Y N N Y N Y</t>
+    <t xml:space="preserve">N N Y N N N Y N N Y N Y</t>
   </si>
   <si>
     <t>Quasar</t>
   </si>
   <si>
-    <t>yynn nynn nyyn</t>
+    <t xml:space="preserve">yynn nynn nyyn</t>
   </si>
   <si>
     <t>Onyx</t>
   </si>
   <si>
-    <t>NYNN YNYN NYYY</t>
+    <t xml:space="preserve">NYNN YNYN NYYY</t>
   </si>
   <si>
     <t>Guduman</t>
   </si>
   <si>
-    <t>YNNN YNNN NNYY</t>
+    <t xml:space="preserve">YNNN YNNN NNYY</t>
   </si>
   <si>
     <t>Lesunal</t>
   </si>
   <si>
-    <t>YYN N NNN N YYN N</t>
-  </si>
-  <si>
-    <t>a very very happy (mat)</t>
+    <t xml:space="preserve">YYN N NNN N YYN N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a very very happy (mat)</t>
   </si>
   <si>
     <t>blee2k</t>
@@ -262,19 +267,19 @@
     <t>Cent</t>
   </si>
   <si>
-    <t>YYNY YNNY NNYN</t>
-  </si>
-  <si>
-    <t>Story Analyst</t>
-  </si>
-  <si>
-    <t>YYNN YNNN NNYN</t>
+    <t xml:space="preserve">YYNY YNNY NNYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Story Analyst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYNN YNNN NNYN</t>
   </si>
   <si>
     <t>SpilledThoughts</t>
   </si>
   <si>
-    <t>NYNN YNYN NYNN</t>
+    <t xml:space="preserve">NYNN YNYN NYNN</t>
   </si>
   <si>
     <t>PERMABANNED</t>
@@ -283,48 +288,48 @@
     <t>MOSH</t>
   </si>
   <si>
-    <t>YNNN YNYN NYYN</t>
+    <t xml:space="preserve">YNNN YNYN NYYN</t>
   </si>
   <si>
     <t>kinora</t>
   </si>
   <si>
-    <t>NYNN YNNN NYYN</t>
+    <t xml:space="preserve">NYNN YNNN NYYN</t>
   </si>
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="17"/>
+        <color rgb="FFC27C0E"/>
         <rFont val="Microsoft YaHei"/>
-        <b/>
-        <color rgb="FFC27C0E"/>
-        <sz val="17.0"/>
       </rPr>
       <t>綾けい</t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="17"/>
+        <color rgb="FFC27C0E"/>
         <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFC27C0E"/>
-        <sz val="17.0"/>
       </rPr>
       <t>(Ayakei)</t>
     </r>
   </si>
   <si>
-    <t>YYY Y YNY N NYY Y</t>
+    <t xml:space="preserve">YYY Y YNY N NYY Y</t>
   </si>
   <si>
     <t>Mand</t>
   </si>
   <si>
-    <t>NNYN NNYN NYNY</t>
+    <t xml:space="preserve">NNYN NNYN NYNY</t>
   </si>
   <si>
     <t>Crom</t>
   </si>
   <si>
-    <t>NYYN NNNN NYYN</t>
+    <t xml:space="preserve">NYYN NNNN NYYN</t>
   </si>
   <si>
     <t>Donten</t>
@@ -333,281 +338,281 @@
     <t>Meraxes</t>
   </si>
   <si>
-    <t>Kallavans Koochie</t>
-  </si>
-  <si>
-    <t>yynn ynnn nyyn</t>
-  </si>
-  <si>
-    <t>Dr. Pro-Pain Man</t>
-  </si>
-  <si>
-    <t>Tubbo Bubbo</t>
+    <t xml:space="preserve">Kallavans Koochie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yynn ynnn nyyn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Pro-Pain Man</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tubbo Bubbo</t>
   </si>
   <si>
     <t>Eddiead</t>
   </si>
   <si>
-    <t>Y Y N Y N N Y N N Y Y N</t>
+    <t xml:space="preserve">Y Y N Y N N Y N N Y Y N</t>
   </si>
   <si>
     <t xml:space="preserve">BadHabit | ANTI - F A T </t>
   </si>
   <si>
-    <t>gustang vs traum</t>
-  </si>
-  <si>
-    <t>NNNY YNNY NYNN</t>
-  </si>
-  <si>
-    <t>Rasengan Bro</t>
-  </si>
-  <si>
-    <t>NNYN YNYY NYNY</t>
+    <t xml:space="preserve">gustang vs traum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNNY YNNY NYNN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rasengan Bro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNYN YNYY NYNY</t>
   </si>
   <si>
     <t>Lightprayer</t>
   </si>
   <si>
-    <t>YNNN NNNN NYYN</t>
+    <t xml:space="preserve">YNNN NNNN NYYN</t>
   </si>
   <si>
     <t>SoulSoil</t>
   </si>
   <si>
-    <t>NYYN YNYN NYYY</t>
+    <t xml:space="preserve">NYYN YNYN NYYY</t>
   </si>
   <si>
     <t xml:space="preserve">ZapZap Æ </t>
   </si>
   <si>
-    <t>YNNY NNNN NYYN</t>
-  </si>
-  <si>
-    <t>1080p PandaHour stan</t>
-  </si>
-  <si>
-    <t>YNNN NNNN NYNN</t>
+    <t xml:space="preserve">YNNY NNNN NYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1080p PandaHour stan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YNNN NNNN NYNN</t>
   </si>
   <si>
     <t>Kaiser</t>
   </si>
   <si>
-    <t>YNNN NNNN NNYN</t>
+    <t xml:space="preserve">YNNN NNNN NNYN</t>
   </si>
   <si>
     <t>WhoIsWho?</t>
   </si>
   <si>
-    <t>YYYN YNYY NYYN</t>
+    <t xml:space="preserve">YYYN YNYY NYYN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="34">
     <font>
-      <sz val="11.0"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFE0CC8D"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12.000000"/>
       <color rgb="FF3F3F3F"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFCA2424"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFBB8C60"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF1ABC9C"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFACB172"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFFF6506"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
+      <color indexed="2"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="17.000000"/>
       <color rgb="FF891BFA"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF59805C"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFC27C0E"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFE75252"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF8DAAC4"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFAC0000"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF7592F0"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF94C2C0"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF07D3D3"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFE91E63"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFF1DF81"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFAA8C2B"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF08E46F"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <u/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF891BFA"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFCCA87F"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF4949DD"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFE87F8D"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFC4D8F8"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFFF69B4"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFC27C0E"/>
       <name val="Microsoft YaHei"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF413DB5"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF111111"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFB9E2C0"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF6AC054"/>
       <name val="Arial"/>
     </font>
@@ -617,136 +622,427 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="36">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="29" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="30" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="31" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="32" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="33" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="8" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="9" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="10" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="11" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="12" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="13" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="14" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="15" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="16" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="17" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="18" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="19" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="20" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="21" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="22" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="23" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="24" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="25" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="26" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="27" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="28" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="29" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="30" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="31" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="32" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="33" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -803,7 +1099,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -829,7 +1125,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -906,7 +1202,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -936,23 +1232,25 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="57.0"/>
-    <col customWidth="1" min="2" max="2" width="38.0"/>
+    <col customWidth="1" min="1" max="1" width="57"/>
+    <col customWidth="1" min="2" max="2" width="38"/>
     <col customWidth="1" min="3" max="3" width="11.57"/>
-    <col customWidth="1" min="4" max="26" width="8.71"/>
+    <col customWidth="1" min="4" max="26" width="8.7100000000000009"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1">
+    <row r="1" ht="21.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -960,7 +1258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1">
+    <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -968,7 +1266,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1">
+    <row r="3" ht="21.75" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -976,7 +1274,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="1">
+    <row r="4" ht="21.75" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
@@ -984,7 +1282,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" ht="14.25" customHeight="1">
+    <row r="5" ht="21.75" customHeight="1">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
@@ -992,7 +1290,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" ht="14.25" customHeight="1">
+    <row r="6" ht="21.75" customHeight="1">
       <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
@@ -1000,7 +1298,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="14.25" customHeight="1">
+    <row r="7" ht="21.75" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
@@ -1008,7 +1306,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="14.25" customHeight="1">
+    <row r="8" ht="21.75" customHeight="1">
       <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
@@ -1016,7 +1314,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" ht="14.25" customHeight="1">
+    <row r="9" ht="21.75" customHeight="1">
       <c r="A9" s="8" t="s">
         <v>15</v>
       </c>
@@ -1024,7 +1322,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" ht="14.25" customHeight="1">
+    <row r="10" ht="21.75" customHeight="1">
       <c r="A10" s="10" t="s">
         <v>17</v>
       </c>
@@ -1032,7 +1330,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" ht="14.25" customHeight="1">
+    <row r="11" ht="21.75" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>19</v>
       </c>
@@ -1040,7 +1338,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" ht="14.25" customHeight="1">
+    <row r="12" ht="21.75" customHeight="1">
       <c r="A12" s="12" t="s">
         <v>21</v>
       </c>
@@ -1048,7 +1346,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" ht="14.25" customHeight="1">
+    <row r="13" ht="21.75" customHeight="1">
       <c r="A13" s="5" t="s">
         <v>23</v>
       </c>
@@ -1056,7 +1354,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" ht="14.25" customHeight="1">
+    <row r="14" ht="21.75" customHeight="1">
       <c r="A14" s="13" t="s">
         <v>25</v>
       </c>
@@ -1064,7 +1362,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" ht="14.25" customHeight="1">
+    <row r="15" ht="21.75" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>27</v>
       </c>
@@ -1072,7 +1370,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" ht="14.25" customHeight="1">
+    <row r="16" ht="21.75" customHeight="1">
       <c r="A16" s="11" t="s">
         <v>29</v>
       </c>
@@ -1080,7 +1378,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" ht="14.25" customHeight="1">
+    <row r="17" ht="21.75" customHeight="1">
       <c r="A17" s="15" t="s">
         <v>31</v>
       </c>
@@ -1088,7 +1386,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" ht="14.25" customHeight="1">
+    <row r="18" ht="21.75" customHeight="1">
       <c r="A18" s="16" t="s">
         <v>33</v>
       </c>
@@ -1096,7 +1394,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" ht="14.25" customHeight="1">
+    <row r="19" ht="21.75" customHeight="1">
       <c r="A19" s="17" t="s">
         <v>35</v>
       </c>
@@ -1104,7 +1402,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" ht="14.25" customHeight="1">
+    <row r="20" ht="21.75" customHeight="1">
       <c r="A20" s="12" t="s">
         <v>37</v>
       </c>
@@ -1112,7 +1410,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" ht="14.25" customHeight="1">
+    <row r="21" ht="21.75" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>39</v>
       </c>
@@ -1120,7 +1418,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" ht="14.25" customHeight="1">
+    <row r="22" ht="21.75" customHeight="1">
       <c r="A22" s="18" t="s">
         <v>41</v>
       </c>
@@ -1128,7 +1426,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" ht="14.25" customHeight="1">
+    <row r="23" ht="21.75" customHeight="1">
       <c r="A23" s="13" t="s">
         <v>43</v>
       </c>
@@ -1136,7 +1434,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" ht="14.25" customHeight="1">
+    <row r="24" ht="21.75" customHeight="1">
       <c r="A24" s="13" t="s">
         <v>45</v>
       </c>
@@ -1144,7 +1442,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="25" ht="14.25" customHeight="1">
+    <row r="25" ht="21.75" customHeight="1">
       <c r="A25" s="5" t="s">
         <v>47</v>
       </c>
@@ -1152,7 +1450,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" ht="14.25" customHeight="1">
+    <row r="26" ht="21.75" customHeight="1">
       <c r="A26" s="19" t="s">
         <v>48</v>
       </c>
@@ -1160,7 +1458,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="27" ht="14.25" customHeight="1">
+    <row r="27" ht="21.75" customHeight="1">
       <c r="A27" s="20" t="s">
         <v>50</v>
       </c>
@@ -1168,7 +1466,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="28" ht="14.25" customHeight="1">
+    <row r="28" ht="21.75" customHeight="1">
       <c r="A28" s="21" t="s">
         <v>52</v>
       </c>
@@ -1176,7 +1474,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="29" ht="14.25" customHeight="1">
+    <row r="29" ht="21.75" customHeight="1">
       <c r="A29" s="22" t="s">
         <v>54</v>
       </c>
@@ -1184,7 +1482,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="30" ht="14.25" customHeight="1">
+    <row r="30" ht="21.75" customHeight="1">
       <c r="A30" s="23" t="s">
         <v>56</v>
       </c>
@@ -1192,7 +1490,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" ht="14.25" customHeight="1">
+    <row r="31" ht="21.75" customHeight="1">
       <c r="A31" s="23" t="s">
         <v>58</v>
       </c>
@@ -1200,7 +1498,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" ht="14.25" customHeight="1">
+    <row r="32" ht="21.75" customHeight="1">
       <c r="A32" s="13" t="s">
         <v>60</v>
       </c>
@@ -1208,7 +1506,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="33" ht="14.25" customHeight="1">
+    <row r="33" ht="21.75" customHeight="1">
       <c r="A33" s="18" t="s">
         <v>62</v>
       </c>
@@ -1216,7 +1514,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="34" ht="14.25" customHeight="1">
+    <row r="34" ht="21.75" customHeight="1">
       <c r="A34" s="4" t="s">
         <v>64</v>
       </c>
@@ -1224,7 +1522,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="35" ht="14.25" customHeight="1">
+    <row r="35" ht="21.75" customHeight="1">
       <c r="A35" s="13" t="s">
         <v>66</v>
       </c>
@@ -1232,7 +1530,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="36" ht="14.25" customHeight="1">
+    <row r="36" ht="21.75" customHeight="1">
       <c r="A36" s="24" t="s">
         <v>68</v>
       </c>
@@ -1240,7 +1538,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="37" ht="14.25" customHeight="1">
+    <row r="37" ht="21.75" customHeight="1">
       <c r="A37" s="20" t="s">
         <v>70</v>
       </c>
@@ -1248,7 +1546,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="38" ht="14.25" customHeight="1">
+    <row r="38" ht="21.75" customHeight="1">
       <c r="A38" s="5" t="s">
         <v>72</v>
       </c>
@@ -1256,7 +1554,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="39" ht="14.25" customHeight="1">
+    <row r="39" ht="21.75" customHeight="1">
       <c r="A39" s="25" t="s">
         <v>74</v>
       </c>
@@ -1264,7 +1562,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="40" ht="14.25" customHeight="1">
+    <row r="40" ht="21.75" customHeight="1">
       <c r="A40" s="26" t="s">
         <v>76</v>
       </c>
@@ -1272,7 +1570,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="41" ht="14.25" customHeight="1">
+    <row r="41" ht="21.75" customHeight="1">
       <c r="A41" s="27" t="s">
         <v>78</v>
       </c>
@@ -1280,7 +1578,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="42" ht="14.25" customHeight="1">
+    <row r="42" ht="21.75" customHeight="1">
       <c r="A42" s="22" t="s">
         <v>80</v>
       </c>
@@ -1288,7 +1586,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="43" ht="14.25" customHeight="1">
+    <row r="43" ht="21.75" customHeight="1">
       <c r="A43" s="8" t="s">
         <v>81</v>
       </c>
@@ -1296,7 +1594,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="44" ht="14.25" customHeight="1">
+    <row r="44" ht="21.75" customHeight="1">
       <c r="A44" s="28" t="s">
         <v>82</v>
       </c>
@@ -1304,7 +1602,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="45" ht="14.25" customHeight="1">
+    <row r="45" ht="21.75" customHeight="1">
       <c r="A45" s="5" t="s">
         <v>84</v>
       </c>
@@ -1312,7 +1610,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="46" ht="14.25" customHeight="1">
+    <row r="46" ht="21.75" customHeight="1">
       <c r="A46" s="29" t="s">
         <v>86</v>
       </c>
@@ -1320,7 +1618,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="47" ht="14.25" customHeight="1">
+    <row r="47" ht="21.75" customHeight="1">
       <c r="A47" s="17" t="s">
         <v>88</v>
       </c>
@@ -1328,7 +1626,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="48" ht="14.25" customHeight="1">
+    <row r="48" ht="21.75" customHeight="1">
       <c r="A48" s="26" t="s">
         <v>89</v>
       </c>
@@ -1336,7 +1634,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" ht="14.25" customHeight="1">
+    <row r="49" ht="21.75" customHeight="1">
       <c r="A49" s="30" t="s">
         <v>91</v>
       </c>
@@ -1344,7 +1642,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="50" ht="14.25" customHeight="1">
+    <row r="50" ht="21.75" customHeight="1">
       <c r="A50" s="31" t="s">
         <v>93</v>
       </c>
@@ -1352,7 +1650,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="51" ht="14.25" customHeight="1">
+    <row r="51" ht="21.75" customHeight="1">
       <c r="A51" s="32" t="s">
         <v>95</v>
       </c>
@@ -1360,7 +1658,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="52" ht="14.25" customHeight="1">
+    <row r="52" ht="21.75" customHeight="1">
       <c r="A52" s="33" t="s">
         <v>97</v>
       </c>
@@ -1368,7 +1666,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="53" ht="14.25" customHeight="1">
+    <row r="53" ht="21.75" customHeight="1">
       <c r="A53" s="34" t="s">
         <v>99</v>
       </c>
@@ -1376,7 +1674,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="54" ht="14.25" customHeight="1">
+    <row r="54" ht="21.75" customHeight="1">
       <c r="A54" s="20" t="s">
         <v>100</v>
       </c>
@@ -1384,7 +1682,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="55" ht="14.25" customHeight="1">
+    <row r="55" ht="21.75" customHeight="1">
       <c r="A55" s="29" t="s">
         <v>101</v>
       </c>
@@ -1392,7 +1690,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="56" ht="14.25" customHeight="1">
+    <row r="56" ht="21.75" customHeight="1">
       <c r="A56" s="35" t="s">
         <v>103</v>
       </c>
@@ -1400,7 +1698,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="57" ht="14.25" customHeight="1">
+    <row r="57" ht="21.75" customHeight="1">
       <c r="A57" s="28" t="s">
         <v>104</v>
       </c>
@@ -1408,7 +1706,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="58" ht="14.25" customHeight="1">
+    <row r="58" ht="21.75" customHeight="1">
       <c r="A58" s="5" t="s">
         <v>105</v>
       </c>
@@ -1416,7 +1714,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="59" ht="14.25" customHeight="1">
+    <row r="59" ht="21.75" customHeight="1">
       <c r="A59" s="34" t="s">
         <v>107</v>
       </c>
@@ -1424,7 +1722,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="60" ht="14.25" customHeight="1">
+    <row r="60" ht="21.75" customHeight="1">
       <c r="A60" s="16" t="s">
         <v>108</v>
       </c>
@@ -1432,7 +1730,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="61" ht="14.25" customHeight="1">
+    <row r="61" ht="21.75" customHeight="1">
       <c r="A61" s="28" t="s">
         <v>110</v>
       </c>
@@ -1440,7 +1738,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="62" ht="14.25" customHeight="1">
+    <row r="62" ht="21.75" customHeight="1">
       <c r="A62" s="16" t="s">
         <v>112</v>
       </c>
@@ -1448,7 +1746,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="63" ht="14.25" customHeight="1">
+    <row r="63" ht="21.75" customHeight="1">
       <c r="A63" s="4" t="s">
         <v>114</v>
       </c>
@@ -1456,7 +1754,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="64" ht="14.25" customHeight="1">
+    <row r="64" ht="21.75" customHeight="1">
       <c r="A64" s="1" t="s">
         <v>116</v>
       </c>
@@ -1464,7 +1762,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="65" ht="14.25" customHeight="1">
+    <row r="65" ht="21.75" customHeight="1">
       <c r="A65" s="1" t="s">
         <v>118</v>
       </c>
@@ -1472,7 +1770,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="66" ht="14.25" customHeight="1">
+    <row r="66" ht="21.75" customHeight="1">
       <c r="A66" s="8" t="s">
         <v>120</v>
       </c>
@@ -1480,7 +1778,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="67" ht="14.25" customHeight="1">
+    <row r="67" ht="21.75" customHeight="1">
       <c r="A67" s="15" t="s">
         <v>122</v>
       </c>
@@ -2422,9 +2720,9 @@
     <row r="999" ht="14.25" customHeight="1"/>
     <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.752083333333333" footer="0.0" header="0.0" left="0.7006944444444448" right="0.7006944444444448" top="0.752083333333333"/>
-  <pageSetup orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70069444444444484" right="0.70069444444444484" top="0.75208333333333299" bottom="0.75208333333333299" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: change bg color to a darker shade (#13)
</commit_message>
<xml_diff>
--- a/tests/128/128.xlsx
+++ b/tests/128/128.xlsx
@@ -1,58 +1,63 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="124">
-  <si>
-    <t>Kobeni Hour</t>
-  </si>
-  <si>
-    <t>YYY Y YNN N NYY Y</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
+  <si>
+    <t xml:space="preserve">Kobeni Hour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYY Y YNN N NYY Y</t>
   </si>
   <si>
     <t>Nomad</t>
   </si>
   <si>
-    <t>N Y N N  N N N N  N Y N N</t>
+    <t xml:space="preserve">N Y N N  N N N N  N Y N N</t>
   </si>
   <si>
     <t>Golden</t>
   </si>
   <si>
-    <t>YYNY YNNN NNYN</t>
+    <t xml:space="preserve">YYNY YNNN NNYN</t>
   </si>
   <si>
     <t>naian77</t>
   </si>
   <si>
-    <t>YYNN YNNN YNYN</t>
-  </si>
-  <si>
-    <t>Daniel Gacitua</t>
-  </si>
-  <si>
-    <t>YYNY NNNN YYYN</t>
-  </si>
-  <si>
-    <t>Urek vs Macseth | Rolo</t>
-  </si>
-  <si>
-    <t>NNNN NNNN NYYN</t>
-  </si>
-  <si>
-    <t>Po Bi D. Au</t>
-  </si>
-  <si>
-    <t>NYNY YNNN NYYN</t>
+    <t xml:space="preserve">YYNN YNNN YNYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daniel Gacitua</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYNY NNNN YYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Urek vs Macseth | Rolo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNNN NNNN NYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Po Bi D. Au</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYNY YNNN NYYN</t>
   </si>
   <si>
     <t>LaFa</t>
@@ -61,199 +66,199 @@
     <t>Jain_friend69</t>
   </si>
   <si>
-    <t>Y Y N N    Y N N Y      Y Y N Y</t>
+    <t xml:space="preserve">Y Y N N    Y N N Y      Y Y N Y</t>
   </si>
   <si>
     <t>Kanika_em</t>
   </si>
   <si>
-    <t>YYNY NNNN NNYN</t>
+    <t xml:space="preserve">YYNY NNNN NNYN</t>
   </si>
   <si>
     <t>hajro</t>
   </si>
   <si>
-    <t>YYYN YNNY NYYN</t>
-  </si>
-  <si>
-    <t>Peak-A-Boo | FATE</t>
-  </si>
-  <si>
-    <t>YNNN YNNY NYYN</t>
+    <t xml:space="preserve">YYYN YNNY NYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peak-A-Boo | FATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YNNN YNNY NYYN</t>
   </si>
   <si>
     <t>Muddy</t>
   </si>
   <si>
-    <t>YYYN YNNY YYYN</t>
+    <t xml:space="preserve">YYYN YNNY YYYN</t>
   </si>
   <si>
     <t>Karneval</t>
   </si>
   <si>
-    <t>YYNN YNNN YYYN</t>
-  </si>
-  <si>
-    <t>Ranker BaamZahard</t>
-  </si>
-  <si>
-    <t>YYNN NNNN NNYY</t>
+    <t xml:space="preserve">YYNN YNNN YYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ranker BaamZahard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYNN NNNN NNYY</t>
   </si>
   <si>
     <t>Ozymanbruh</t>
   </si>
   <si>
-    <t>YNYY YYNN YYYN</t>
-  </si>
-  <si>
-    <t>Griot | ♾</t>
-  </si>
-  <si>
-    <t>NNYN YNNN NYNY</t>
+    <t xml:space="preserve">YNYY YYNN YYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Griot | ♾</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNYN YNNN NYNY</t>
   </si>
   <si>
     <t>malts</t>
   </si>
   <si>
-    <t>YYYN NNNN NYYY</t>
+    <t xml:space="preserve">YYYN NNNN NYYY</t>
   </si>
   <si>
     <t>Eggroll6996</t>
   </si>
   <si>
-    <t>NYNN NNNN NYYN</t>
+    <t xml:space="preserve">NYNN NNNN NYYN</t>
   </si>
   <si>
     <t>Hatikva</t>
   </si>
   <si>
-    <t>YYNN YNYN NYYN</t>
+    <t xml:space="preserve">YYNN YNYN NYYN</t>
   </si>
   <si>
     <t>Eiheir</t>
   </si>
   <si>
-    <t>YYN Y YNN N NYY Y</t>
-  </si>
-  <si>
-    <t>colorless june</t>
-  </si>
-  <si>
-    <t>NNYY YNYN NYNN</t>
+    <t xml:space="preserve">YYN Y YNN N NYY Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">colorless june</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNYY YNYN NYNN</t>
   </si>
   <si>
     <t>RajaBranco</t>
   </si>
   <si>
-    <t>YYNN YNNN NYYN</t>
+    <t xml:space="preserve">YYNN YNNN NYYN</t>
   </si>
   <si>
     <t>Saint</t>
   </si>
   <si>
-    <t>YYYN YNYY  YNYN</t>
-  </si>
-  <si>
-    <t>Best girl For sure</t>
+    <t xml:space="preserve">YYYN YNYY  YNYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best girl For sure</t>
   </si>
   <si>
     <t>Headon's🍆Heaven</t>
   </si>
   <si>
-    <t>NYYN YNYY NYNN</t>
-  </si>
-  <si>
-    <t>Rodeosquad 👑| Son Of Ari</t>
-  </si>
-  <si>
-    <t>YNNY YNNN NYYN</t>
+    <t xml:space="preserve">NYYN YNYY NYNN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rodeosquad 👑| Son Of Ari</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YNNY YNNN NYYN</t>
   </si>
   <si>
     <t>Platon</t>
   </si>
   <si>
-    <t>YYNY YNNN NYYN</t>
-  </si>
-  <si>
-    <t>Thien | thicc thighs save lives</t>
-  </si>
-  <si>
-    <t>YYNN NNNN NYYN</t>
-  </si>
-  <si>
-    <t>Amr Ahmed | Jinsung supremacy |</t>
-  </si>
-  <si>
-    <t>YYYY YNYY YYYY</t>
-  </si>
-  <si>
-    <t>Jinsung fanboy</t>
-  </si>
-  <si>
-    <t>NNNN NNNN NNNN</t>
+    <t xml:space="preserve">YYNY YNNN NYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thien | thicc thighs save lives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYNN NNNN NYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amr Ahmed | Jinsung supremacy |</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYYY YNYY YYYY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jinsung fanboy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNNN NNNN NNNN</t>
   </si>
   <si>
     <t>SirLordBoss</t>
   </si>
   <si>
-    <t>YYYY YYYY NYNN</t>
+    <t xml:space="preserve">YYYY YYYY NYNN</t>
   </si>
   <si>
     <t>Sathya</t>
   </si>
   <si>
-    <t>YYYY YYYY YYYY</t>
+    <t xml:space="preserve">YYYY YYYY YYYY</t>
   </si>
   <si>
     <t>Naronu</t>
   </si>
   <si>
-    <t>Y Y N N Y N N Y Y N Y N</t>
+    <t xml:space="preserve">Y Y N N Y N N Y Y N Y N</t>
   </si>
   <si>
     <t>Popcorn</t>
   </si>
   <si>
-    <t>NNNN YNNN YYYN</t>
+    <t xml:space="preserve">NNNN YNNN YYYN</t>
   </si>
   <si>
     <t>Lopobiasimp</t>
   </si>
   <si>
-    <t>NNNY YNYN NYNN</t>
+    <t xml:space="preserve">NNNY YNYN NYNN</t>
   </si>
   <si>
     <t>RTSK0929</t>
   </si>
   <si>
-    <t>N N Y N N N Y N N Y N Y</t>
+    <t xml:space="preserve">N N Y N N N Y N N Y N Y</t>
   </si>
   <si>
     <t>Quasar</t>
   </si>
   <si>
-    <t>yynn nynn nyyn</t>
+    <t xml:space="preserve">yynn nynn nyyn</t>
   </si>
   <si>
     <t>Onyx</t>
   </si>
   <si>
-    <t>NYNN YNYN NYYY</t>
+    <t xml:space="preserve">NYNN YNYN NYYY</t>
   </si>
   <si>
     <t>Guduman</t>
   </si>
   <si>
-    <t>YNNN YNNN NNYY</t>
+    <t xml:space="preserve">YNNN YNNN NNYY</t>
   </si>
   <si>
     <t>Lesunal</t>
   </si>
   <si>
-    <t>YYN N NNN N YYN N</t>
-  </si>
-  <si>
-    <t>a very very happy (mat)</t>
+    <t xml:space="preserve">YYN N NNN N YYN N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a very very happy (mat)</t>
   </si>
   <si>
     <t>blee2k</t>
@@ -262,19 +267,19 @@
     <t>Cent</t>
   </si>
   <si>
-    <t>YYNY YNNY NNYN</t>
-  </si>
-  <si>
-    <t>Story Analyst</t>
-  </si>
-  <si>
-    <t>YYNN YNNN NNYN</t>
+    <t xml:space="preserve">YYNY YNNY NNYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Story Analyst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YYNN YNNN NNYN</t>
   </si>
   <si>
     <t>SpilledThoughts</t>
   </si>
   <si>
-    <t>NYNN YNYN NYNN</t>
+    <t xml:space="preserve">NYNN YNYN NYNN</t>
   </si>
   <si>
     <t>PERMABANNED</t>
@@ -283,48 +288,48 @@
     <t>MOSH</t>
   </si>
   <si>
-    <t>YNNN YNYN NYYN</t>
+    <t xml:space="preserve">YNNN YNYN NYYN</t>
   </si>
   <si>
     <t>kinora</t>
   </si>
   <si>
-    <t>NYNN YNNN NYYN</t>
+    <t xml:space="preserve">NYNN YNNN NYYN</t>
   </si>
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="17"/>
+        <color rgb="FFC27C0E"/>
         <rFont val="Microsoft YaHei"/>
-        <b/>
-        <color rgb="FFC27C0E"/>
-        <sz val="17.0"/>
       </rPr>
       <t>綾けい</t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="17"/>
+        <color rgb="FFC27C0E"/>
         <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFC27C0E"/>
-        <sz val="17.0"/>
       </rPr>
       <t>(Ayakei)</t>
     </r>
   </si>
   <si>
-    <t>YYY Y YNY N NYY Y</t>
+    <t xml:space="preserve">YYY Y YNY N NYY Y</t>
   </si>
   <si>
     <t>Mand</t>
   </si>
   <si>
-    <t>NNYN NNYN NYNY</t>
+    <t xml:space="preserve">NNYN NNYN NYNY</t>
   </si>
   <si>
     <t>Crom</t>
   </si>
   <si>
-    <t>NYYN NNNN NYYN</t>
+    <t xml:space="preserve">NYYN NNNN NYYN</t>
   </si>
   <si>
     <t>Donten</t>
@@ -333,281 +338,281 @@
     <t>Meraxes</t>
   </si>
   <si>
-    <t>Kallavans Koochie</t>
-  </si>
-  <si>
-    <t>yynn ynnn nyyn</t>
-  </si>
-  <si>
-    <t>Dr. Pro-Pain Man</t>
-  </si>
-  <si>
-    <t>Tubbo Bubbo</t>
+    <t xml:space="preserve">Kallavans Koochie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yynn ynnn nyyn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dr. Pro-Pain Man</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tubbo Bubbo</t>
   </si>
   <si>
     <t>Eddiead</t>
   </si>
   <si>
-    <t>Y Y N Y N N Y N N Y Y N</t>
+    <t xml:space="preserve">Y Y N Y N N Y N N Y Y N</t>
   </si>
   <si>
     <t xml:space="preserve">BadHabit | ANTI - F A T </t>
   </si>
   <si>
-    <t>gustang vs traum</t>
-  </si>
-  <si>
-    <t>NNNY YNNY NYNN</t>
-  </si>
-  <si>
-    <t>Rasengan Bro</t>
-  </si>
-  <si>
-    <t>NNYN YNYY NYNY</t>
+    <t xml:space="preserve">gustang vs traum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNNY YNNY NYNN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rasengan Bro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NNYN YNYY NYNY</t>
   </si>
   <si>
     <t>Lightprayer</t>
   </si>
   <si>
-    <t>YNNN NNNN NYYN</t>
+    <t xml:space="preserve">YNNN NNNN NYYN</t>
   </si>
   <si>
     <t>SoulSoil</t>
   </si>
   <si>
-    <t>NYYN YNYN NYYY</t>
+    <t xml:space="preserve">NYYN YNYN NYYY</t>
   </si>
   <si>
     <t xml:space="preserve">ZapZap Æ </t>
   </si>
   <si>
-    <t>YNNY NNNN NYYN</t>
-  </si>
-  <si>
-    <t>1080p PandaHour stan</t>
-  </si>
-  <si>
-    <t>YNNN NNNN NYNN</t>
+    <t xml:space="preserve">YNNY NNNN NYYN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1080p PandaHour stan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YNNN NNNN NYNN</t>
   </si>
   <si>
     <t>Kaiser</t>
   </si>
   <si>
-    <t>YNNN NNNN NNYN</t>
+    <t xml:space="preserve">YNNN NNNN NNYN</t>
   </si>
   <si>
     <t>WhoIsWho?</t>
   </si>
   <si>
-    <t>YYYN YNYY NYYN</t>
+    <t xml:space="preserve">YYYN YNYY NYYN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="34">
     <font>
-      <sz val="11.0"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFE0CC8D"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12.000000"/>
       <color rgb="FF3F3F3F"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFCA2424"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFBB8C60"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF1ABC9C"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFACB172"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFFF6506"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
+      <color indexed="2"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="17.000000"/>
       <color rgb="FF891BFA"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF59805C"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFC27C0E"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFE75252"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF8DAAC4"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFAC0000"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF7592F0"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF94C2C0"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF07D3D3"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFE91E63"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFF1DF81"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFAA8C2B"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF08E46F"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <u/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF891BFA"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFCCA87F"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF4949DD"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFE87F8D"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFC4D8F8"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFFF69B4"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFC27C0E"/>
       <name val="Microsoft YaHei"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF413DB5"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF111111"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FFB9E2C0"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="17.0"/>
+      <sz val="17.000000"/>
       <color rgb="FF6AC054"/>
       <name val="Arial"/>
     </font>
@@ -617,136 +622,427 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="36">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="19" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="24" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="25" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="28" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="29" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="30" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="31" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="32" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="33" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="8" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="9" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="10" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="11" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="12" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="13" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="14" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="15" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="16" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="17" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="18" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="19" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="20" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="21" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="22" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="23" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="24" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="25" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="26" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="27" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="28" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="29" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="30" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="31" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="32" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="33" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -803,7 +1099,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -829,7 +1125,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -906,7 +1202,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -936,23 +1232,25 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="57.0"/>
-    <col customWidth="1" min="2" max="2" width="38.0"/>
+    <col customWidth="1" min="1" max="1" width="57"/>
+    <col customWidth="1" min="2" max="2" width="38"/>
     <col customWidth="1" min="3" max="3" width="11.57"/>
-    <col customWidth="1" min="4" max="26" width="8.71"/>
+    <col customWidth="1" min="4" max="26" width="8.7100000000000009"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1">
+    <row r="1" ht="21.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -960,7 +1258,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1">
+    <row r="2" ht="21.75" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -968,7 +1266,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1">
+    <row r="3" ht="21.75" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -976,7 +1274,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="1">
+    <row r="4" ht="21.75" customHeight="1">
       <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
@@ -984,7 +1282,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" ht="14.25" customHeight="1">
+    <row r="5" ht="21.75" customHeight="1">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
@@ -992,7 +1290,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" ht="14.25" customHeight="1">
+    <row r="6" ht="21.75" customHeight="1">
       <c r="A6" s="6" t="s">
         <v>10</v>
       </c>
@@ -1000,7 +1298,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" ht="14.25" customHeight="1">
+    <row r="7" ht="21.75" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
@@ -1008,7 +1306,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" ht="14.25" customHeight="1">
+    <row r="8" ht="21.75" customHeight="1">
       <c r="A8" s="7" t="s">
         <v>14</v>
       </c>
@@ -1016,7 +1314,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" ht="14.25" customHeight="1">
+    <row r="9" ht="21.75" customHeight="1">
       <c r="A9" s="8" t="s">
         <v>15</v>
       </c>
@@ -1024,7 +1322,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" ht="14.25" customHeight="1">
+    <row r="10" ht="21.75" customHeight="1">
       <c r="A10" s="10" t="s">
         <v>17</v>
       </c>
@@ -1032,7 +1330,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" ht="14.25" customHeight="1">
+    <row r="11" ht="21.75" customHeight="1">
       <c r="A11" s="11" t="s">
         <v>19</v>
       </c>
@@ -1040,7 +1338,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" ht="14.25" customHeight="1">
+    <row r="12" ht="21.75" customHeight="1">
       <c r="A12" s="12" t="s">
         <v>21</v>
       </c>
@@ -1048,7 +1346,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" ht="14.25" customHeight="1">
+    <row r="13" ht="21.75" customHeight="1">
       <c r="A13" s="5" t="s">
         <v>23</v>
       </c>
@@ -1056,7 +1354,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" ht="14.25" customHeight="1">
+    <row r="14" ht="21.75" customHeight="1">
       <c r="A14" s="13" t="s">
         <v>25</v>
       </c>
@@ -1064,7 +1362,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" ht="14.25" customHeight="1">
+    <row r="15" ht="21.75" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>27</v>
       </c>
@@ -1072,7 +1370,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" ht="14.25" customHeight="1">
+    <row r="16" ht="21.75" customHeight="1">
       <c r="A16" s="11" t="s">
         <v>29</v>
       </c>
@@ -1080,7 +1378,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" ht="14.25" customHeight="1">
+    <row r="17" ht="21.75" customHeight="1">
       <c r="A17" s="15" t="s">
         <v>31</v>
       </c>
@@ -1088,7 +1386,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" ht="14.25" customHeight="1">
+    <row r="18" ht="21.75" customHeight="1">
       <c r="A18" s="16" t="s">
         <v>33</v>
       </c>
@@ -1096,7 +1394,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" ht="14.25" customHeight="1">
+    <row r="19" ht="21.75" customHeight="1">
       <c r="A19" s="17" t="s">
         <v>35</v>
       </c>
@@ -1104,7 +1402,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="20" ht="14.25" customHeight="1">
+    <row r="20" ht="21.75" customHeight="1">
       <c r="A20" s="12" t="s">
         <v>37</v>
       </c>
@@ -1112,7 +1410,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" ht="14.25" customHeight="1">
+    <row r="21" ht="21.75" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>39</v>
       </c>
@@ -1120,7 +1418,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="22" ht="14.25" customHeight="1">
+    <row r="22" ht="21.75" customHeight="1">
       <c r="A22" s="18" t="s">
         <v>41</v>
       </c>
@@ -1128,7 +1426,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" ht="14.25" customHeight="1">
+    <row r="23" ht="21.75" customHeight="1">
       <c r="A23" s="13" t="s">
         <v>43</v>
       </c>
@@ -1136,7 +1434,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" ht="14.25" customHeight="1">
+    <row r="24" ht="21.75" customHeight="1">
       <c r="A24" s="13" t="s">
         <v>45</v>
       </c>
@@ -1144,7 +1442,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="25" ht="14.25" customHeight="1">
+    <row r="25" ht="21.75" customHeight="1">
       <c r="A25" s="5" t="s">
         <v>47</v>
       </c>
@@ -1152,7 +1450,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="26" ht="14.25" customHeight="1">
+    <row r="26" ht="21.75" customHeight="1">
       <c r="A26" s="19" t="s">
         <v>48</v>
       </c>
@@ -1160,7 +1458,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="27" ht="14.25" customHeight="1">
+    <row r="27" ht="21.75" customHeight="1">
       <c r="A27" s="20" t="s">
         <v>50</v>
       </c>
@@ -1168,7 +1466,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="28" ht="14.25" customHeight="1">
+    <row r="28" ht="21.75" customHeight="1">
       <c r="A28" s="21" t="s">
         <v>52</v>
       </c>
@@ -1176,7 +1474,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="29" ht="14.25" customHeight="1">
+    <row r="29" ht="21.75" customHeight="1">
       <c r="A29" s="22" t="s">
         <v>54</v>
       </c>
@@ -1184,7 +1482,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="30" ht="14.25" customHeight="1">
+    <row r="30" ht="21.75" customHeight="1">
       <c r="A30" s="23" t="s">
         <v>56</v>
       </c>
@@ -1192,7 +1490,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" ht="14.25" customHeight="1">
+    <row r="31" ht="21.75" customHeight="1">
       <c r="A31" s="23" t="s">
         <v>58</v>
       </c>
@@ -1200,7 +1498,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" ht="14.25" customHeight="1">
+    <row r="32" ht="21.75" customHeight="1">
       <c r="A32" s="13" t="s">
         <v>60</v>
       </c>
@@ -1208,7 +1506,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="33" ht="14.25" customHeight="1">
+    <row r="33" ht="21.75" customHeight="1">
       <c r="A33" s="18" t="s">
         <v>62</v>
       </c>
@@ -1216,7 +1514,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="34" ht="14.25" customHeight="1">
+    <row r="34" ht="21.75" customHeight="1">
       <c r="A34" s="4" t="s">
         <v>64</v>
       </c>
@@ -1224,7 +1522,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="35" ht="14.25" customHeight="1">
+    <row r="35" ht="21.75" customHeight="1">
       <c r="A35" s="13" t="s">
         <v>66</v>
       </c>
@@ -1232,7 +1530,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="36" ht="14.25" customHeight="1">
+    <row r="36" ht="21.75" customHeight="1">
       <c r="A36" s="24" t="s">
         <v>68</v>
       </c>
@@ -1240,7 +1538,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="37" ht="14.25" customHeight="1">
+    <row r="37" ht="21.75" customHeight="1">
       <c r="A37" s="20" t="s">
         <v>70</v>
       </c>
@@ -1248,7 +1546,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="38" ht="14.25" customHeight="1">
+    <row r="38" ht="21.75" customHeight="1">
       <c r="A38" s="5" t="s">
         <v>72</v>
       </c>
@@ -1256,7 +1554,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="39" ht="14.25" customHeight="1">
+    <row r="39" ht="21.75" customHeight="1">
       <c r="A39" s="25" t="s">
         <v>74</v>
       </c>
@@ -1264,7 +1562,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="40" ht="14.25" customHeight="1">
+    <row r="40" ht="21.75" customHeight="1">
       <c r="A40" s="26" t="s">
         <v>76</v>
       </c>
@@ -1272,7 +1570,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="41" ht="14.25" customHeight="1">
+    <row r="41" ht="21.75" customHeight="1">
       <c r="A41" s="27" t="s">
         <v>78</v>
       </c>
@@ -1280,7 +1578,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="42" ht="14.25" customHeight="1">
+    <row r="42" ht="21.75" customHeight="1">
       <c r="A42" s="22" t="s">
         <v>80</v>
       </c>
@@ -1288,7 +1586,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="43" ht="14.25" customHeight="1">
+    <row r="43" ht="21.75" customHeight="1">
       <c r="A43" s="8" t="s">
         <v>81</v>
       </c>
@@ -1296,7 +1594,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="44" ht="14.25" customHeight="1">
+    <row r="44" ht="21.75" customHeight="1">
       <c r="A44" s="28" t="s">
         <v>82</v>
       </c>
@@ -1304,7 +1602,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="45" ht="14.25" customHeight="1">
+    <row r="45" ht="21.75" customHeight="1">
       <c r="A45" s="5" t="s">
         <v>84</v>
       </c>
@@ -1312,7 +1610,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="46" ht="14.25" customHeight="1">
+    <row r="46" ht="21.75" customHeight="1">
       <c r="A46" s="29" t="s">
         <v>86</v>
       </c>
@@ -1320,7 +1618,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="47" ht="14.25" customHeight="1">
+    <row r="47" ht="21.75" customHeight="1">
       <c r="A47" s="17" t="s">
         <v>88</v>
       </c>
@@ -1328,7 +1626,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="48" ht="14.25" customHeight="1">
+    <row r="48" ht="21.75" customHeight="1">
       <c r="A48" s="26" t="s">
         <v>89</v>
       </c>
@@ -1336,7 +1634,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="49" ht="14.25" customHeight="1">
+    <row r="49" ht="21.75" customHeight="1">
       <c r="A49" s="30" t="s">
         <v>91</v>
       </c>
@@ -1344,7 +1642,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="50" ht="14.25" customHeight="1">
+    <row r="50" ht="21.75" customHeight="1">
       <c r="A50" s="31" t="s">
         <v>93</v>
       </c>
@@ -1352,7 +1650,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="51" ht="14.25" customHeight="1">
+    <row r="51" ht="21.75" customHeight="1">
       <c r="A51" s="32" t="s">
         <v>95</v>
       </c>
@@ -1360,7 +1658,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="52" ht="14.25" customHeight="1">
+    <row r="52" ht="21.75" customHeight="1">
       <c r="A52" s="33" t="s">
         <v>97</v>
       </c>
@@ -1368,7 +1666,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="53" ht="14.25" customHeight="1">
+    <row r="53" ht="21.75" customHeight="1">
       <c r="A53" s="34" t="s">
         <v>99</v>
       </c>
@@ -1376,7 +1674,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="54" ht="14.25" customHeight="1">
+    <row r="54" ht="21.75" customHeight="1">
       <c r="A54" s="20" t="s">
         <v>100</v>
       </c>
@@ -1384,7 +1682,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="55" ht="14.25" customHeight="1">
+    <row r="55" ht="21.75" customHeight="1">
       <c r="A55" s="29" t="s">
         <v>101</v>
       </c>
@@ -1392,7 +1690,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="56" ht="14.25" customHeight="1">
+    <row r="56" ht="21.75" customHeight="1">
       <c r="A56" s="35" t="s">
         <v>103</v>
       </c>
@@ -1400,7 +1698,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="57" ht="14.25" customHeight="1">
+    <row r="57" ht="21.75" customHeight="1">
       <c r="A57" s="28" t="s">
         <v>104</v>
       </c>
@@ -1408,7 +1706,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="58" ht="14.25" customHeight="1">
+    <row r="58" ht="21.75" customHeight="1">
       <c r="A58" s="5" t="s">
         <v>105</v>
       </c>
@@ -1416,7 +1714,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="59" ht="14.25" customHeight="1">
+    <row r="59" ht="21.75" customHeight="1">
       <c r="A59" s="34" t="s">
         <v>107</v>
       </c>
@@ -1424,7 +1722,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="60" ht="14.25" customHeight="1">
+    <row r="60" ht="21.75" customHeight="1">
       <c r="A60" s="16" t="s">
         <v>108</v>
       </c>
@@ -1432,7 +1730,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="61" ht="14.25" customHeight="1">
+    <row r="61" ht="21.75" customHeight="1">
       <c r="A61" s="28" t="s">
         <v>110</v>
       </c>
@@ -1440,7 +1738,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="62" ht="14.25" customHeight="1">
+    <row r="62" ht="21.75" customHeight="1">
       <c r="A62" s="16" t="s">
         <v>112</v>
       </c>
@@ -1448,7 +1746,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="63" ht="14.25" customHeight="1">
+    <row r="63" ht="21.75" customHeight="1">
       <c r="A63" s="4" t="s">
         <v>114</v>
       </c>
@@ -1456,7 +1754,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="64" ht="14.25" customHeight="1">
+    <row r="64" ht="21.75" customHeight="1">
       <c r="A64" s="1" t="s">
         <v>116</v>
       </c>
@@ -1464,7 +1762,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="65" ht="14.25" customHeight="1">
+    <row r="65" ht="21.75" customHeight="1">
       <c r="A65" s="1" t="s">
         <v>118</v>
       </c>
@@ -1472,7 +1770,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="66" ht="14.25" customHeight="1">
+    <row r="66" ht="21.75" customHeight="1">
       <c r="A66" s="8" t="s">
         <v>120</v>
       </c>
@@ -1480,7 +1778,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="67" ht="14.25" customHeight="1">
+    <row r="67" ht="21.75" customHeight="1">
       <c r="A67" s="15" t="s">
         <v>122</v>
       </c>
@@ -2422,9 +2720,9 @@
     <row r="999" ht="14.25" customHeight="1"/>
     <row r="1000" ht="14.25" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.752083333333333" footer="0.0" header="0.0" left="0.7006944444444448" right="0.7006944444444448" top="0.752083333333333"/>
-  <pageSetup orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70069444444444484" right="0.70069444444444484" top="0.75208333333333299" bottom="0.75208333333333299" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>